<commit_message>
changes made to lbv_first fig in slides
</commit_message>
<xml_diff>
--- a/icfd2026/pres/figures/lbv_num_phi-10.xlsx
+++ b/icfd2026/pres/figures/lbv_num_phi-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rgd\Documents\lab\presentation\icfd2026\pres\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F41D6CC-F851-4D89-BE2C-DF497D1A1FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D97F6D-C9F6-4869-9626-643D526F9AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8A2922A7-97E9-46A4-AC71-0CE1B71449A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>xh2</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Okafor Reduced 2019</t>
+  </si>
+  <si>
+    <t>Okafor Detailed 2018</t>
   </si>
 </sst>
 </file>
@@ -86,8 +89,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,10 +427,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88D1EA39-B5A2-4371-984E-74D79CF4BC8C}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -437,10 +441,13 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -450,11 +457,14 @@
       <c r="C2" s="1">
         <v>6.4339079999999997</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
+        <v>7.0059389999999997</v>
+      </c>
+      <c r="E2" s="1">
         <v>7.4488539999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0.2</v>
       </c>
@@ -464,11 +474,14 @@
       <c r="C3" s="1">
         <v>10.412240000000001</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
+        <v>11.62951</v>
+      </c>
+      <c r="E3" s="1">
         <v>13.356490000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>0.4</v>
       </c>
@@ -478,11 +491,14 @@
       <c r="C4" s="1">
         <v>18.608969999999999</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
+        <v>21.866689999999998</v>
+      </c>
+      <c r="E4" s="1">
         <v>26.882930000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>0.6</v>
       </c>
@@ -492,11 +508,14 @@
       <c r="C5" s="1">
         <v>39.131570000000004</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
+        <v>49.450049999999997</v>
+      </c>
+      <c r="E5" s="1">
         <v>61.796320000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>0.8</v>
       </c>
@@ -506,9 +525,15 @@
       <c r="C6" s="1">
         <v>93.56335</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
+        <v>108.5256</v>
+      </c>
+      <c r="E6" s="1">
         <v>129.47819999999999</v>
       </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>